<commit_message>
D: intake of A's 64 manually downloaded OA PDFs (DOI-verified; 2 swapped records corrected); 4 still pending
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fulltext_requests/library_requests_2026-10-09.xlsx
+++ b/fulltext_requests/library_requests_2026-10-09.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="library_not_OA" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="not_indexed" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="browser_OA_D_will_fetch" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="browser_OA_64_done_4_pending" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,12 +38,17 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF59D"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -59,10 +64,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -573,7 +580,6 @@
           <t>FS-007033.pdf</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -634,7 +640,6 @@
           <t>FS-006499.pdf</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -695,7 +700,6 @@
           <t>FS-006366.pdf</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -756,7 +760,6 @@
           <t>FS-006410.pdf</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -817,7 +820,6 @@
           <t>FS-005607.pdf</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -878,7 +880,6 @@
           <t>FS-008737.pdf</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -939,7 +940,6 @@
           <t>FS-004989.pdf</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1000,7 +1000,6 @@
           <t>FS-004769.pdf</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1061,7 +1060,6 @@
           <t>FS-004839.pdf</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1122,7 +1120,6 @@
           <t>FS-004724.pdf</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1183,7 +1180,6 @@
           <t>FS-004147.pdf</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1244,7 +1240,6 @@
           <t>FS-004390.pdf</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1305,7 +1300,6 @@
           <t>FS-004179.pdf</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1366,7 +1360,6 @@
           <t>FS-003901.pdf</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1427,7 +1420,6 @@
           <t>FS-004098.pdf</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1488,7 +1480,6 @@
           <t>FS-003691.pdf</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1549,7 +1540,6 @@
           <t>FS-003468.pdf</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1610,7 +1600,6 @@
           <t>FS-003532.pdf</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1671,7 +1660,6 @@
           <t>FS-003800.pdf</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1732,7 +1720,6 @@
           <t>FS-003615.pdf</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1793,7 +1780,6 @@
           <t>FS-003210.pdf</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1854,7 +1840,6 @@
           <t>FS-003254.pdf</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1915,7 +1900,6 @@
           <t>FS-003108.pdf</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1976,7 +1960,6 @@
           <t>FS-002589.pdf</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2037,7 +2020,6 @@
           <t>FS-002569.pdf</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2098,7 +2080,6 @@
           <t>FS-002764.pdf</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2159,7 +2140,6 @@
           <t>FS-002327.pdf</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2220,7 +2200,6 @@
           <t>FS-002265.pdf</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2281,7 +2260,6 @@
           <t>FS-010465.pdf</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2342,7 +2320,6 @@
           <t>FS-002021.pdf</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2403,7 +2380,6 @@
           <t>FS-001575.pdf</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2464,7 +2440,6 @@
           <t>FS-001835.pdf</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2525,7 +2500,6 @@
           <t>FS-001489.pdf</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2586,7 +2560,6 @@
           <t>FS-001733.pdf</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2647,7 +2620,6 @@
           <t>FS-001612.pdf</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2708,7 +2680,6 @@
           <t>FS-001622.pdf</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2769,7 +2740,6 @@
           <t>FS-001364.pdf</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2830,7 +2800,6 @@
           <t>FS-001536.pdf</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2891,7 +2860,6 @@
           <t>FS-001197.pdf</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2952,7 +2920,6 @@
           <t>FS-001324.pdf</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3013,7 +2980,6 @@
           <t>FS-001370.pdf</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3074,7 +3040,6 @@
           <t>FS-001117.pdf</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3135,7 +3100,6 @@
           <t>FS-001140.pdf</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3196,7 +3160,6 @@
           <t>FS-001207.pdf</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3257,7 +3220,6 @@
           <t>FS-001039.pdf</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3283,13 +3245,11 @@
           <t>2006</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>16596116</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
       <c r="I47" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/16596116/</t>
@@ -3310,7 +3270,6 @@
           <t>FS-000951.pdf</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3371,7 +3330,6 @@
           <t>FS-000829.pdf</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3432,7 +3390,6 @@
           <t>FS-000837.pdf</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3493,7 +3450,6 @@
           <t>FS-000873.pdf</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3554,7 +3510,6 @@
           <t>FS-000885.pdf</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3615,7 +3570,6 @@
           <t>FS-000693.pdf</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3641,13 +3595,11 @@
           <t>2004</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>15756172</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
       <c r="I53" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/15756172/</t>
@@ -3668,7 +3620,6 @@
           <t>FS-000751.pdf</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3729,7 +3680,6 @@
           <t>FS-000533.pdf</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3790,7 +3740,6 @@
           <t>FS-000451.pdf</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3851,7 +3800,6 @@
           <t>FS-000472.pdf</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3912,7 +3860,6 @@
           <t>FS-011327.pdf</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3973,7 +3920,6 @@
           <t>FS-000404.pdf</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4034,7 +3980,6 @@
           <t>FS-000297.pdf</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -4095,7 +4040,6 @@
           <t>FS-000287.pdf</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -4156,7 +4100,6 @@
           <t>FS-000212.pdf</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -4217,7 +4160,6 @@
           <t>FS-000242.pdf</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4278,7 +4220,6 @@
           <t>FS-000102.pdf</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -4339,7 +4280,6 @@
           <t>FS-000106.pdf</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -4400,7 +4340,6 @@
           <t>FS-000142.pdf</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -4461,7 +4400,6 @@
           <t>FS-000156.pdf</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -4522,7 +4460,6 @@
           <t>FS-007778.pdf</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -4583,7 +4520,6 @@
           <t>FS-007801.pdf</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -4644,7 +4580,6 @@
           <t>FS-007508.pdf</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -4675,13 +4610,11 @@
           <t>10.1136/bjsm.29.1.61</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
       <c r="H70" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1136/bjsm.29.1.61</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
       <c r="J70" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1136/bjsm.29.1.61</t>
@@ -4697,7 +4630,6 @@
           <t>FS-013865.pdf</t>
         </is>
       </c>
-      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -4758,7 +4690,6 @@
           <t>FS-007479.pdf</t>
         </is>
       </c>
-      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -4819,7 +4750,6 @@
           <t>FS-007641.pdf</t>
         </is>
       </c>
-      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -4880,7 +4810,6 @@
           <t>FS-007530.pdf</t>
         </is>
       </c>
-      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -4941,7 +4870,6 @@
           <t>FS-007565.pdf</t>
         </is>
       </c>
-      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -5002,7 +4930,6 @@
           <t>FS-007578.pdf</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -5063,7 +4990,6 @@
           <t>FS-000573.pdf</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -5124,7 +5050,6 @@
           <t>FS-002301.pdf</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -5150,13 +5075,11 @@
           <t>1988</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>3375945</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/3375945/</t>
@@ -5177,7 +5100,6 @@
           <t>FS-005118.pdf</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -5238,7 +5160,6 @@
           <t>FS-007440.pdf</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -5299,7 +5220,6 @@
           <t>FS-000266.pdf</t>
         </is>
       </c>
-      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -5360,7 +5280,6 @@
           <t>FS-006949.pdf</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -5421,7 +5340,6 @@
           <t>FS-006965.pdf</t>
         </is>
       </c>
-      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -5482,7 +5400,6 @@
           <t>FS-007100.pdf</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -5543,7 +5460,6 @@
           <t>FS-007188.pdf</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -5604,7 +5520,6 @@
           <t>FS-007236.pdf</t>
         </is>
       </c>
-      <c r="M85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -5665,7 +5580,6 @@
           <t>FS-007308.pdf</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -5726,7 +5640,6 @@
           <t>FS-006563.pdf</t>
         </is>
       </c>
-      <c r="M87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -5787,7 +5700,6 @@
           <t>FS-006651.pdf</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -5848,7 +5760,6 @@
           <t>FS-006706.pdf</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -5909,7 +5820,6 @@
           <t>FS-006734.pdf</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -5970,7 +5880,6 @@
           <t>FS-006154.pdf</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -6031,7 +5940,6 @@
           <t>FS-006184.pdf</t>
         </is>
       </c>
-      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -6092,7 +6000,6 @@
           <t>FS-006215.pdf</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -6153,7 +6060,6 @@
           <t>FS-006260.pdf</t>
         </is>
       </c>
-      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -6214,7 +6120,6 @@
           <t>FS-006296.pdf</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -6275,7 +6180,6 @@
           <t>FS-006373.pdf</t>
         </is>
       </c>
-      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -6336,7 +6240,6 @@
           <t>FS-005434.pdf</t>
         </is>
       </c>
-      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -6397,7 +6300,6 @@
           <t>FS-005856.pdf</t>
         </is>
       </c>
-      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -6458,7 +6360,6 @@
           <t>FS-005334.pdf</t>
         </is>
       </c>
-      <c r="M99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -6519,7 +6420,6 @@
           <t>FS-005183.pdf</t>
         </is>
       </c>
-      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -6580,7 +6480,6 @@
           <t>FS-004509.pdf</t>
         </is>
       </c>
-      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -6641,7 +6540,6 @@
           <t>FS-004231.pdf</t>
         </is>
       </c>
-      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -6702,7 +6600,6 @@
           <t>FS-004116.pdf</t>
         </is>
       </c>
-      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -6763,7 +6660,6 @@
           <t>FS-003581.pdf</t>
         </is>
       </c>
-      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -6824,7 +6720,6 @@
           <t>FS-003838.pdf</t>
         </is>
       </c>
-      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -6885,7 +6780,6 @@
           <t>FS-003209.pdf</t>
         </is>
       </c>
-      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -6946,7 +6840,6 @@
           <t>FS-003073.pdf</t>
         </is>
       </c>
-      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -7007,7 +6900,6 @@
           <t>FS-002618.pdf</t>
         </is>
       </c>
-      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -7068,7 +6960,6 @@
           <t>FS-002619.pdf</t>
         </is>
       </c>
-      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -7129,7 +7020,6 @@
           <t>FS-002638.pdf</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -7190,7 +7080,6 @@
           <t>FS-002666.pdf</t>
         </is>
       </c>
-      <c r="M111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -7251,7 +7140,6 @@
           <t>FS-002669.pdf</t>
         </is>
       </c>
-      <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -7277,13 +7165,11 @@
           <t>2014</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>25316129</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
       <c r="I113" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/25316129/</t>
@@ -7304,7 +7190,6 @@
           <t>FS-002878.pdf</t>
         </is>
       </c>
-      <c r="M113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -7365,7 +7250,6 @@
           <t>FS-002346.pdf</t>
         </is>
       </c>
-      <c r="M114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -7426,7 +7310,6 @@
           <t>FS-002421.pdf</t>
         </is>
       </c>
-      <c r="M115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -7487,7 +7370,6 @@
           <t>FS-002435.pdf</t>
         </is>
       </c>
-      <c r="M116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -7548,7 +7430,6 @@
           <t>FS-002554.pdf</t>
         </is>
       </c>
-      <c r="M117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -7609,7 +7490,6 @@
           <t>FS-001994.pdf</t>
         </is>
       </c>
-      <c r="M118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -7670,7 +7550,6 @@
           <t>FS-002059.pdf</t>
         </is>
       </c>
-      <c r="M119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -7731,7 +7610,6 @@
           <t>FS-002156.pdf</t>
         </is>
       </c>
-      <c r="M120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -7792,7 +7670,6 @@
           <t>FS-002241.pdf</t>
         </is>
       </c>
-      <c r="M121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -7818,13 +7695,11 @@
           <t>2012</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>22846291</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
       <c r="I122" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/22846291/</t>
@@ -7845,7 +7720,6 @@
           <t>FS-010564.pdf</t>
         </is>
       </c>
-      <c r="M122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -7906,7 +7780,6 @@
           <t>FS-001918.pdf</t>
         </is>
       </c>
-      <c r="M123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -7967,7 +7840,6 @@
           <t>FS-001987.pdf</t>
         </is>
       </c>
-      <c r="M124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -8028,7 +7900,6 @@
           <t>FS-002032.pdf</t>
         </is>
       </c>
-      <c r="M125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -8089,7 +7960,6 @@
           <t>FS-001584.pdf</t>
         </is>
       </c>
-      <c r="M126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -8150,7 +8020,6 @@
           <t>FS-001595.pdf</t>
         </is>
       </c>
-      <c r="M127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -8211,7 +8080,6 @@
           <t>FS-001615.pdf</t>
         </is>
       </c>
-      <c r="M128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -8272,7 +8140,6 @@
           <t>FS-001635.pdf</t>
         </is>
       </c>
-      <c r="M129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -8333,7 +8200,6 @@
           <t>FS-001211.pdf</t>
         </is>
       </c>
-      <c r="M130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -8394,7 +8260,6 @@
           <t>FS-001024.pdf</t>
         </is>
       </c>
-      <c r="M131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -8455,7 +8320,6 @@
           <t>FS-000816.pdf</t>
         </is>
       </c>
-      <c r="M132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -8516,7 +8380,6 @@
           <t>FS-000645.pdf</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -8577,7 +8440,6 @@
           <t>FS-000319.pdf</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -8638,7 +8500,6 @@
           <t>FS-000182.pdf</t>
         </is>
       </c>
-      <c r="M135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -8699,7 +8560,6 @@
           <t>FS-006885.pdf</t>
         </is>
       </c>
-      <c r="M136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -8760,7 +8620,6 @@
           <t>FS-007097.pdf</t>
         </is>
       </c>
-      <c r="M137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -8821,7 +8680,6 @@
           <t>FS-007241.pdf</t>
         </is>
       </c>
-      <c r="M138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -8882,7 +8740,6 @@
           <t>FS-007259.pdf</t>
         </is>
       </c>
-      <c r="M139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -8943,7 +8800,6 @@
           <t>FS-007330.pdf</t>
         </is>
       </c>
-      <c r="M140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -9004,7 +8860,6 @@
           <t>FS-006114.pdf</t>
         </is>
       </c>
-      <c r="M141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -9065,7 +8920,6 @@
           <t>FS-006172.pdf</t>
         </is>
       </c>
-      <c r="M142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -9126,7 +8980,6 @@
           <t>FS-006462.pdf</t>
         </is>
       </c>
-      <c r="M143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -9187,7 +9040,6 @@
           <t>FS-008584.pdf</t>
         </is>
       </c>
-      <c r="M144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -9248,7 +9100,6 @@
           <t>FS-004666.pdf</t>
         </is>
       </c>
-      <c r="M145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -9274,13 +9125,11 @@
           <t>2022</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
           <t>32619204</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/32619204/</t>
@@ -9301,7 +9150,6 @@
           <t>FS-004809.pdf</t>
         </is>
       </c>
-      <c r="M146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -9362,7 +9210,6 @@
           <t>FS-005508.pdf</t>
         </is>
       </c>
-      <c r="M147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -9423,7 +9270,6 @@
           <t>FS-004773.pdf</t>
         </is>
       </c>
-      <c r="M148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -9484,7 +9330,6 @@
           <t>FS-004819.pdf</t>
         </is>
       </c>
-      <c r="M149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -9545,7 +9390,6 @@
           <t>FS-004954.pdf</t>
         </is>
       </c>
-      <c r="M150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -9606,7 +9450,6 @@
           <t>FS-005169.pdf</t>
         </is>
       </c>
-      <c r="M151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -9632,13 +9475,11 @@
           <t>2021</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
           <t>34543566</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
       <c r="I152" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/34543566/</t>
@@ -9659,7 +9500,6 @@
           <t>FS-005304.pdf</t>
         </is>
       </c>
-      <c r="M152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -9720,7 +9560,6 @@
           <t>FS-004518.pdf</t>
         </is>
       </c>
-      <c r="M153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -9781,7 +9620,6 @@
           <t>FS-004537.pdf</t>
         </is>
       </c>
-      <c r="M154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -9842,7 +9680,6 @@
           <t>FS-004568.pdf</t>
         </is>
       </c>
-      <c r="M155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -9903,7 +9740,6 @@
           <t>FS-004580.pdf</t>
         </is>
       </c>
-      <c r="M156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -9964,7 +9800,6 @@
           <t>FS-004083.pdf</t>
         </is>
       </c>
-      <c r="M157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -10025,7 +9860,6 @@
           <t>FS-004138.pdf</t>
         </is>
       </c>
-      <c r="M158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -10086,7 +9920,6 @@
           <t>FS-004154.pdf</t>
         </is>
       </c>
-      <c r="M159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -10147,7 +9980,6 @@
           <t>FS-004361.pdf</t>
         </is>
       </c>
-      <c r="M160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -10208,7 +10040,6 @@
           <t>FS-003815.pdf</t>
         </is>
       </c>
-      <c r="M161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -10269,7 +10100,6 @@
           <t>FS-003879.pdf</t>
         </is>
       </c>
-      <c r="M162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -10330,7 +10160,6 @@
           <t>FS-003943.pdf</t>
         </is>
       </c>
-      <c r="M163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -10391,7 +10220,6 @@
           <t>FS-009343.pdf</t>
         </is>
       </c>
-      <c r="M164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -10452,7 +10280,6 @@
           <t>FS-003642.pdf</t>
         </is>
       </c>
-      <c r="M165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -10513,7 +10340,6 @@
           <t>FS-003783.pdf</t>
         </is>
       </c>
-      <c r="M166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -10574,7 +10400,6 @@
           <t>FS-003840.pdf</t>
         </is>
       </c>
-      <c r="M167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -10635,7 +10460,6 @@
           <t>FS-009525.pdf</t>
         </is>
       </c>
-      <c r="M168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -10696,7 +10520,6 @@
           <t>FS-002641.pdf</t>
         </is>
       </c>
-      <c r="M169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -10757,7 +10580,6 @@
           <t>FS-003173.pdf</t>
         </is>
       </c>
-      <c r="M170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -10818,7 +10640,6 @@
           <t>FS-003224.pdf</t>
         </is>
       </c>
-      <c r="M171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -10879,7 +10700,6 @@
           <t>FS-003274.pdf</t>
         </is>
       </c>
-      <c r="M172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -10940,7 +10760,6 @@
           <t>FS-003334.pdf</t>
         </is>
       </c>
-      <c r="M173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -11001,7 +10820,6 @@
           <t>FS-002803.pdf</t>
         </is>
       </c>
-      <c r="M174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -11062,7 +10880,6 @@
           <t>FS-002906.pdf</t>
         </is>
       </c>
-      <c r="M175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -11123,7 +10940,6 @@
           <t>FS-002940.pdf</t>
         </is>
       </c>
-      <c r="M176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -11184,7 +11000,6 @@
           <t>FS-002948.pdf</t>
         </is>
       </c>
-      <c r="M177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -11245,7 +11060,6 @@
           <t>FS-003030.pdf</t>
         </is>
       </c>
-      <c r="M178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -11306,7 +11120,6 @@
           <t>FS-002841.pdf</t>
         </is>
       </c>
-      <c r="M179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -11367,7 +11180,6 @@
           <t>FS-010114.pdf</t>
         </is>
       </c>
-      <c r="M180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -11428,7 +11240,6 @@
           <t>FS-002511.pdf</t>
         </is>
       </c>
-      <c r="M181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -11489,7 +11300,6 @@
           <t>FS-010351.pdf</t>
         </is>
       </c>
-      <c r="M182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -11550,7 +11360,6 @@
           <t>FS-002071.pdf</t>
         </is>
       </c>
-      <c r="M183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -11611,7 +11420,6 @@
           <t>FS-002077.pdf</t>
         </is>
       </c>
-      <c r="M184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -11672,7 +11480,6 @@
           <t>FS-002079.pdf</t>
         </is>
       </c>
-      <c r="M185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -11733,7 +11540,6 @@
           <t>FS-002172.pdf</t>
         </is>
       </c>
-      <c r="M186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -11794,7 +11600,6 @@
           <t>FS-002180.pdf</t>
         </is>
       </c>
-      <c r="M187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -11855,7 +11660,6 @@
           <t>FS-010516.pdf</t>
         </is>
       </c>
-      <c r="M188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -11916,7 +11720,6 @@
           <t>FS-001833.pdf</t>
         </is>
       </c>
-      <c r="M189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -11942,13 +11745,11 @@
           <t>2011</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
           <t>22212276</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr"/>
       <c r="I190" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/22212276/</t>
@@ -11969,7 +11770,6 @@
           <t>FS-002088.pdf</t>
         </is>
       </c>
-      <c r="M190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -12030,7 +11830,6 @@
           <t>FS-001310.pdf</t>
         </is>
       </c>
-      <c r="M191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -12091,7 +11890,6 @@
           <t>FS-001598.pdf</t>
         </is>
       </c>
-      <c r="M192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -12152,7 +11950,6 @@
           <t>FS-001505.pdf</t>
         </is>
       </c>
-      <c r="M193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -12178,13 +11975,11 @@
           <t>2009</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
           <t>24149537</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr"/>
       <c r="I194" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/24149537/</t>
@@ -12205,7 +12000,6 @@
           <t>FS-002573.pdf</t>
         </is>
       </c>
-      <c r="M194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -12231,13 +12025,11 @@
           <t>2009</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr">
         <is>
           <t>24149602</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr"/>
       <c r="I195" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/24149602/</t>
@@ -12258,7 +12050,6 @@
           <t>FS-002578.pdf</t>
         </is>
       </c>
-      <c r="M195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -12319,7 +12110,6 @@
           <t>FS-001269.pdf</t>
         </is>
       </c>
-      <c r="M196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -12380,7 +12170,6 @@
           <t>FS-001280.pdf</t>
         </is>
       </c>
-      <c r="M197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -12441,7 +12230,6 @@
           <t>FS-001293.pdf</t>
         </is>
       </c>
-      <c r="M198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -12502,7 +12290,6 @@
           <t>FS-001339.pdf</t>
         </is>
       </c>
-      <c r="M199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -12563,7 +12350,6 @@
           <t>FS-001372.pdf</t>
         </is>
       </c>
-      <c r="M200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -12624,7 +12410,6 @@
           <t>FS-000995.pdf</t>
         </is>
       </c>
-      <c r="M201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -12685,7 +12470,6 @@
           <t>FS-001044.pdf</t>
         </is>
       </c>
-      <c r="M202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -12746,7 +12530,6 @@
           <t>FS-001146.pdf</t>
         </is>
       </c>
-      <c r="M203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -12807,7 +12590,6 @@
           <t>FS-001172.pdf</t>
         </is>
       </c>
-      <c r="M204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -12868,7 +12650,6 @@
           <t>FS-001176.pdf</t>
         </is>
       </c>
-      <c r="M205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -12929,7 +12710,6 @@
           <t>FS-000912.pdf</t>
         </is>
       </c>
-      <c r="M206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -12990,7 +12770,6 @@
           <t>FS-000925.pdf</t>
         </is>
       </c>
-      <c r="M207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -13051,7 +12830,6 @@
           <t>FS-000953.pdf</t>
         </is>
       </c>
-      <c r="M208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -13112,7 +12890,6 @@
           <t>FS-000972.pdf</t>
         </is>
       </c>
-      <c r="M209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -13173,7 +12950,6 @@
           <t>FS-000983.pdf</t>
         </is>
       </c>
-      <c r="M210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -13234,7 +13010,6 @@
           <t>FS-000990.pdf</t>
         </is>
       </c>
-      <c r="M211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -13295,7 +13070,6 @@
           <t>FS-000681.pdf</t>
         </is>
       </c>
-      <c r="M212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -13356,7 +13130,6 @@
           <t>FS-000726.pdf</t>
         </is>
       </c>
-      <c r="M213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -13417,7 +13190,6 @@
           <t>FS-000425.pdf</t>
         </is>
       </c>
-      <c r="M214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -13478,7 +13250,6 @@
           <t>FS-000450.pdf</t>
         </is>
       </c>
-      <c r="M215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -13539,7 +13310,6 @@
           <t>FS-000389.pdf</t>
         </is>
       </c>
-      <c r="M216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -13600,7 +13370,6 @@
           <t>FS-000274.pdf</t>
         </is>
       </c>
-      <c r="M217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -13661,7 +13430,6 @@
           <t>FS-000059.pdf</t>
         </is>
       </c>
-      <c r="M218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -13722,7 +13490,6 @@
           <t>FS-000076.pdf</t>
         </is>
       </c>
-      <c r="M219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -13783,7 +13550,6 @@
           <t>FS-007796.pdf</t>
         </is>
       </c>
-      <c r="M220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -13809,13 +13575,11 @@
           <t>1997</t>
         </is>
       </c>
-      <c r="F221" t="inlineStr"/>
       <c r="G221" t="inlineStr">
         <is>
           <t>9502526</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
       <c r="I221" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/9502526/</t>
@@ -13836,7 +13600,6 @@
           <t>FS-007775.pdf</t>
         </is>
       </c>
-      <c r="M221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -13897,7 +13660,6 @@
           <t>FS-007639.pdf</t>
         </is>
       </c>
-      <c r="M222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -13958,7 +13720,6 @@
           <t>FS-007642.pdf</t>
         </is>
       </c>
-      <c r="M223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -13984,13 +13745,11 @@
           <t>1996</t>
         </is>
       </c>
-      <c r="F224" t="inlineStr"/>
       <c r="G224" t="inlineStr">
         <is>
           <t>8898521</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr"/>
       <c r="I224" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/8898521/</t>
@@ -14011,7 +13770,6 @@
           <t>FS-011807.pdf</t>
         </is>
       </c>
-      <c r="M224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -14072,7 +13830,6 @@
           <t>FS-007501.pdf</t>
         </is>
       </c>
-      <c r="M225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -14103,13 +13860,11 @@
           <t>10.1042/bst023124s</t>
         </is>
       </c>
-      <c r="G226" t="inlineStr"/>
       <c r="H226" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1042/bst023124s</t>
         </is>
       </c>
-      <c r="I226" t="inlineStr"/>
       <c r="J226" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1042/bst023124s</t>
@@ -14125,7 +13880,6 @@
           <t>FS-013867.pdf</t>
         </is>
       </c>
-      <c r="M226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -14186,7 +13940,6 @@
           <t>FS-007528.pdf</t>
         </is>
       </c>
-      <c r="M227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -14247,7 +14000,6 @@
           <t>FS-007602.pdf</t>
         </is>
       </c>
-      <c r="M228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -14308,7 +14060,6 @@
           <t>FS-000719.pdf</t>
         </is>
       </c>
-      <c r="M229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -14369,7 +14120,6 @@
           <t>FS-001904.pdf</t>
         </is>
       </c>
-      <c r="M230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -14430,7 +14180,6 @@
           <t>FS-001905.pdf</t>
         </is>
       </c>
-      <c r="M231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -14456,13 +14205,11 @@
           <t>1983</t>
         </is>
       </c>
-      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
           <t>6408915</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
       <c r="I232" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/6408915/</t>
@@ -14483,7 +14230,6 @@
           <t>FS-007404.pdf</t>
         </is>
       </c>
-      <c r="M232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -14544,7 +14290,6 @@
           <t>FS-007452.pdf</t>
         </is>
       </c>
-      <c r="M233" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -15586,13 +15331,11 @@
           <t>10.4103/bbrj.bbrj_72_26</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.4103/bbrj.bbrj_72_26</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.4103/bbrj.bbrj_72_26</t>
@@ -15608,7 +15351,6 @@
           <t>FS-007953.pdf</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -15639,13 +15381,11 @@
           <t>10.1590/1980-0037.2025v27e99591</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1590/1980-0037.2025v27e99591</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1590/1980-0037.2025v27e99591</t>
@@ -15661,7 +15401,6 @@
           <t>FS-008228.pdf</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -15692,13 +15431,11 @@
           <t>10.2478/pjst-2023-0001</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.2478/pjst-2023-0001</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.2478/pjst-2023-0001</t>
@@ -15714,7 +15451,6 @@
           <t>FS-008738.pdf</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -15745,13 +15481,11 @@
           <t>10.2478/pjst-2021-0014</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.2478/pjst-2021-0014</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.2478/pjst-2021-0014</t>
@@ -15767,7 +15501,6 @@
           <t>FS-008929.pdf</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -15798,13 +15531,11 @@
           <t>10.16926/par.2019.07.11</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.16926/par.2019.07.11</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.16926/par.2019.07.11</t>
@@ -15820,7 +15551,6 @@
           <t>FS-009361.pdf</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -15851,13 +15581,11 @@
           <t>10.1039/c7ay01676j</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1039/c7ay01676j</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1039/c7ay01676j</t>
@@ -15873,7 +15601,6 @@
           <t>FS-009509.pdf</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -15934,7 +15661,6 @@
           <t>FS-003290.pdf</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -15995,7 +15721,6 @@
           <t>FS-002536.pdf</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -16026,13 +15751,11 @@
           <t>10.5604/965481</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.5604/965481</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.5604/965481</t>
@@ -16048,7 +15771,6 @@
           <t>FS-010457.pdf</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -16079,13 +15801,11 @@
           <t>10.1515/JLM.2010.005</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1515/JLM.2010.005</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1515/JLM.2010.005</t>
@@ -16101,7 +15821,6 @@
           <t>FS-010763.pdf</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -16162,7 +15881,6 @@
           <t>FS-001787.pdf</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -16193,13 +15911,11 @@
           <t>10.1016/j.jtherbio.2007.07.001</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jtherbio.2007.07.001</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1016/j.jtherbio.2007.07.001</t>
@@ -16215,7 +15931,6 @@
           <t>FS-011007.pdf</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -16246,13 +15961,11 @@
           <t>10.1515/pteridines.2006.17.4.121</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1515/pteridines.2006.17.4.121</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1515/pteridines.2006.17.4.121</t>
@@ -16268,7 +15981,6 @@
           <t>FS-011033.pdf</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -16294,11 +16006,6 @@
           <t>2004</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Mucosal%20IgA%20response%20to%20intense%20intermittent%20exercise%20in%20healthy%20male%20and%20female%20adults%22</t>
@@ -16309,7 +16016,6 @@
           <t>FS-011064.pdf</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -16340,13 +16046,11 @@
           <t>10.1092/BTWQ5YMYVQ67QK9L</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1092/BTWQ5YMYVQ67QK9L</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1092/BTWQ5YMYVQ67QK9L</t>
@@ -16362,7 +16066,6 @@
           <t>FS-013731.pdf</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -16388,11 +16091,6 @@
           <t>1993</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Temporal%20relationship%20between%20decreased%20salivary%20IgA%20and%20upper%20respiratory%20tract%20infection%20in%20elite%20athletes%22</t>
@@ -16403,7 +16101,6 @@
           <t>FS-011687.pdf</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -16464,7 +16161,6 @@
           <t>FS-007384.pdf</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -16495,13 +16191,11 @@
           <t>10.1016/s0021-8707(37)90440-4</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/s0021-8707(37)90440-4</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1016/s0021-8707(37)90440-4</t>
@@ -16517,7 +16211,6 @@
           <t>FS-013023.pdf</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -16578,7 +16271,6 @@
           <t>FS-006861.pdf</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -16639,7 +16331,6 @@
           <t>FS-004513.pdf</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -16670,13 +16361,11 @@
           <t>10.1016/j.jtherbio.2011.03.013</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jtherbio.2011.03.013</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1016/j.jtherbio.2011.03.013</t>
@@ -16692,7 +16381,6 @@
           <t>FS-010498.pdf</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -16753,7 +16441,6 @@
           <t>FS-000901.pdf</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -16784,13 +16471,11 @@
           <t>10.33275/1727-7485.1.2026.762</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.33275/1727-7485.1.2026.762</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.33275/1727-7485.1.2026.762</t>
@@ -16806,7 +16491,6 @@
           <t>FS-007992.pdf</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -16837,13 +16521,11 @@
           <t>10.3390/app14124968</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/app14124968</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.3390/app14124968</t>
@@ -16859,7 +16541,6 @@
           <t>FS-008227.pdf</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -16890,13 +16571,11 @@
           <t>10.19193/0393-6384_2021_2_168</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.19193/0393-6384_2021_2_168</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.19193/0393-6384_2021_2_168</t>
@@ -16912,7 +16591,6 @@
           <t>FS-009093.pdf</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -16943,13 +16621,11 @@
           <t>10.1177/1747954118779656</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1177/1747954118779656</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1177/1747954118779656</t>
@@ -16965,7 +16641,6 @@
           <t>FS-009341.pdf</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -16996,13 +16671,11 @@
           <t>10.7752/jpes.2018.03259</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.7752/jpes.2018.03259</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.7752/jpes.2018.03259</t>
@@ -17018,7 +16691,6 @@
           <t>FS-009498.pdf</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -17049,13 +16721,11 @@
           <t>10.1590/1517-869220182403171999</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1590/1517-869220182403171999</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1590/1517-869220182403171999</t>
@@ -17071,7 +16741,6 @@
           <t>FS-009520.pdf</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -17102,13 +16771,11 @@
           <t>10.1080/24748668.2018.1501993</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1080/24748668.2018.1501993</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1080/24748668.2018.1501993</t>
@@ -17124,7 +16791,6 @@
           <t>FS-009547.pdf</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -17155,13 +16821,11 @@
           <t>10.2174/1573401313666170725114130</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.2174/1573401313666170725114130</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.2174/1573401313666170725114130</t>
@@ -17177,7 +16841,6 @@
           <t>FS-009633.pdf</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -17208,13 +16871,11 @@
           <t>10.18869/acadpub.aassjournal.4.2.17</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.18869/acadpub.aassjournal.4.2.17</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.18869/acadpub.aassjournal.4.2.17</t>
@@ -17230,7 +16891,6 @@
           <t>FS-013408.pdf</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -17291,7 +16951,6 @@
           <t>FS-003022.pdf</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -17317,11 +16976,6 @@
           <t>2014</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Evaluation%20of%206-month%20periodisation%20in%20male%20ekiden%20runners%20by%20assessment%20of%20muscle%20fatigue%20and%20immune%20function%22</t>
@@ -17332,7 +16986,6 @@
           <t>FS-010165.pdf</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -17363,13 +17016,11 @@
           <t>10.1080/17461391003699070</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1080/17461391003699070</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1080/17461391003699070</t>
@@ -17385,7 +17036,6 @@
           <t>FS-010649.pdf</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -17416,13 +17066,11 @@
           <t>10.5604/20831862.927493</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.5604/20831862.927493</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.5604/20831862.927493</t>
@@ -17438,7 +17086,6 @@
           <t>FS-010740.pdf</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -17464,11 +17111,6 @@
           <t>2010</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Biomedical%20aspects%20of%2051%20consecutive%20marathons%3B%20%5BAspetti%20biomedici%20di%2051%20maratone%20consecutive%5D%22</t>
@@ -17479,7 +17121,6 @@
           <t>FS-010790.pdf</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -17505,11 +17146,6 @@
           <t>2010</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Biomedical%20aspects%20of%2051%20consecutive%20marathons%22</t>
@@ -17520,7 +17156,6 @@
           <t>FS-013573.pdf</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -17551,13 +17186,11 @@
           <t>10.1080/17461390802251844</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1080/17461390802251844</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1080/17461390802251844</t>
@@ -17573,7 +17206,6 @@
           <t>FS-010849.pdf</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -17634,7 +17266,6 @@
           <t>FS-010827.pdf</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -17665,13 +17296,11 @@
           <t>10.1016/j.scispo.2006.09.005</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.scispo.2006.09.005</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1016/j.scispo.2006.09.005</t>
@@ -17687,7 +17316,6 @@
           <t>FS-010873.pdf</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -17748,7 +17376,6 @@
           <t>FS-000731.pdf</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -17774,11 +17401,6 @@
           <t>2003</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
       <c r="K43" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22The%20effects%20of%20eccentric%20exercise-induced%20muscle%20damage%20on%20peripheral%20blood%20neutrophil%20respiratory%20burst%20response%20and%20activation%20status%20in%20humans%22</t>
@@ -17789,7 +17411,6 @@
           <t>FS-015048.pdf</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -17815,11 +17436,6 @@
           <t>2003</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22The%20effect%20of%20exercise-induced%20muscle%20damage%20on%20neutrophil%20function%22</t>
@@ -17830,7 +17446,6 @@
           <t>FS-015049.pdf</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -17856,11 +17471,6 @@
           <t>2002</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Can%20white%20blood%20cell%20activation%20be%20one%20of%20the%20major%20factors%20that%20affect%20hemorheological%20parameters%20during%20and%20after%20exercise%3F%22</t>
@@ -17871,7 +17481,6 @@
           <t>FS-012651.pdf</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -17897,11 +17506,6 @@
           <t>2001</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22The%20adaptable%20change%20of%20the%20function%20of%20T%20lymphocytes%20for%20physical%20exercise%20with%20oxygen%22</t>
@@ -17912,7 +17516,6 @@
           <t>FS-011580.pdf</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -17943,13 +17546,11 @@
           <t>10.12968/bjtr.2000.7.12.13831</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.12968/bjtr.2000.7.12.13831</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
       <c r="J47" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.12968/bjtr.2000.7.12.13831</t>
@@ -17965,7 +17566,6 @@
           <t>FS-011412.pdf</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -17996,13 +17596,11 @@
           <t>10.7600/jspfsm1949.48.147</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.7600/jspfsm1949.48.147</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.7600/jspfsm1949.48.147</t>
@@ -18018,7 +17616,6 @@
           <t>FS-013794.pdf</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -18044,11 +17641,6 @@
           <t>1997</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Acute%20phase%20response%20and%20stress%20related%20hormones%20after%20repeated%20endurance%20exercise%22</t>
@@ -18059,7 +17651,6 @@
           <t>FS-011432.pdf</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -18090,13 +17681,11 @@
           <t>10.1080/15438629009511887</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1080/15438629009511887</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1080/15438629009511887</t>
@@ -18112,7 +17701,6 @@
           <t>FS-011962.pdf</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -18138,11 +17726,6 @@
           <t>1990</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22C-reactive%20protein%20as%20an%20indicator%20of%20post-exercise%20muscle%20damage%22</t>
@@ -18153,7 +17736,6 @@
           <t>FS-011982.pdf</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -18179,11 +17761,6 @@
           <t>1985</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Enhanced%20hydrogen%20peroxide%20generation%20by%20human%20neutrophils%20following%20exercise%22</t>
@@ -18194,7 +17771,6 @@
           <t>FS-011944.pdf</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -18220,11 +17796,6 @@
           <t>1985</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
       <c r="K53" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Correlation%20of%20plasma%20interleukin-1%20%28IL-1%29%20and%20creatine%20kinase%20%28CK%29%20activities%20following%20exercise%22</t>
@@ -18235,7 +17806,6 @@
           <t>FS-012006.pdf</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -18261,11 +17831,6 @@
           <t>1984</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Effect%20of%20acute%20exercise%20on%20immune%20homeostasis%22</t>
@@ -18276,7 +17841,6 @@
           <t>FS-011900.pdf</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -18302,11 +17866,6 @@
           <t>1978</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
       <c r="K55" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Increased%20insulin%20binding%20to%20monocytes%20after%20exercise%3A%20Cellular%20mechanism%20of%20augmented%20insulin%20sensitivity%22</t>
@@ -18317,7 +17876,6 @@
           <t>FS-012067.pdf</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -18618,7 +18176,11 @@
           <t>FS-007251.pdf</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -18679,7 +18241,11 @@
           <t>FS-007158.pdf</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -18740,7 +18306,11 @@
           <t>FS-006824.pdf</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -18801,7 +18371,11 @@
           <t>FS-006681.pdf</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -18862,7 +18436,11 @@
           <t>FS-006745.pdf</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -18923,7 +18501,11 @@
           <t>FS-006828.pdf</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -18984,7 +18566,11 @@
           <t>FS-008442.pdf</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -19045,7 +18631,11 @@
           <t>FS-005160.pdf</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -19106,7 +18696,11 @@
           <t>FS-004624.pdf</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -19167,7 +18761,11 @@
           <t>FS-004640.pdf</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -19228,7 +18826,11 @@
           <t>FS-004719.pdf</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -19289,7 +18891,11 @@
           <t>FS-004798.pdf</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -19350,7 +18956,11 @@
           <t>FS-005046.pdf</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -19411,7 +19021,11 @@
           <t>FS-004193.pdf</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -19472,7 +19086,11 @@
           <t>FS-004303.pdf</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -19533,7 +19151,11 @@
           <t>FS-004349.pdf</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -19594,7 +19216,11 @@
           <t>FS-003808.pdf</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -19655,68 +19281,76 @@
           <t>FS-002374.pdf</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>FS-002317</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Does proteinuria-inducing physical activity increase biomarkers of acute kidney injury?</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Kidney &amp; blood pressure research</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>2012</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>10.1159/000343417</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>23182776</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1159/000343417</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/23182776/</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>https://europepmc.org/article/MED/23182776</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Does%20proteinuria-inducing%20physical%20activity%20increase%20biomarkers%20of%20acute%20kidney%20injury%3F%22</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L20" s="3" t="inlineStr">
         <is>
           <t>FS-002317.pdf</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>PENDING_no_pdf_found</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -19777,68 +19411,76 @@
           <t>FS-001224.pdf</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>FS-000504</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Immune and oxidative changes during and following the Western States Endurance Run.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>International journal of sports medicine</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>2003</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>10.1055/s-2003-42018</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>12968214</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1055/s-2003-42018</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/12968214/</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
         <is>
           <t>https://europepmc.org/article/MED/12968214</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="K22" s="4" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Immune%20and%20oxidative%20changes%20during%20and%20following%20the%20Western%20States%20Endurance%20Run.%22</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L22" s="3" t="inlineStr">
         <is>
           <t>FS-000504.pdf</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>PENDING_no_pdf_found</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -19899,7 +19541,11 @@
           <t>FS-000124.pdf</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -19960,7 +19606,11 @@
           <t>FS-006662.pdf</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -20021,7 +19671,11 @@
           <t>FS-006881.pdf</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -20082,7 +19736,11 @@
           <t>FS-006247.pdf</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -20143,7 +19801,11 @@
           <t>FS-006424.pdf</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -20204,7 +19866,11 @@
           <t>FS-005741.pdf</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -20265,7 +19931,11 @@
           <t>FS-005864.pdf</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -20326,7 +19996,11 @@
           <t>FS-005870.pdf</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -20387,7 +20061,11 @@
           <t>FS-005884.pdf</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -20448,7 +20126,11 @@
           <t>FS-005990.pdf</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -20509,7 +20191,11 @@
           <t>FS-006131.pdf</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -20570,7 +20256,11 @@
           <t>FS-005528.pdf</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -20631,7 +20321,11 @@
           <t>FS-005770.pdf</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -20692,7 +20386,11 @@
           <t>FS-005301.pdf</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -20723,13 +20421,11 @@
           <t>10.3389/fnut.2020.00121</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.3389/fnut.2020.00121</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.3389/fnut.2020.00121</t>
@@ -20745,7 +20441,11 @@
           <t>FS-009203.pdf</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -20806,7 +20506,11 @@
           <t>FS-004374.pdf</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -20867,7 +20571,11 @@
           <t>FS-004392.pdf</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -20928,7 +20636,11 @@
           <t>FS-003994.pdf</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -20989,7 +20701,11 @@
           <t>FS-003556.pdf</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -21050,7 +20766,11 @@
           <t>FS-003475.pdf</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -21111,7 +20831,11 @@
           <t>FS-002635.pdf</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -21172,7 +20896,11 @@
           <t>FS-002742.pdf</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -21233,7 +20961,11 @@
           <t>FS-002283.pdf</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -21294,7 +21026,11 @@
           <t>FS-002123.pdf</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -21355,7 +21091,11 @@
           <t>FS-007201.pdf</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -21416,7 +21156,11 @@
           <t>FS-006191.pdf</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -21477,7 +21221,11 @@
           <t>FS-006439.pdf</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -21538,7 +21286,11 @@
           <t>FS-005887.pdf</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -21599,7 +21351,11 @@
           <t>FS-006008.pdf</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -21660,7 +21416,11 @@
           <t>FS-005701.pdf</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -21721,7 +21481,11 @@
           <t>FS-004889.pdf</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -21782,7 +21546,11 @@
           <t>FS-005129.pdf</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -21843,7 +21611,11 @@
           <t>FS-005337.pdf</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -21904,7 +21676,11 @@
           <t>FS-004269.pdf</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -21935,13 +21711,11 @@
           <t>10.1002/tsm2.23</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/tsm2.23</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
       <c r="J57" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.1002/tsm2.23</t>
@@ -21957,60 +21731,68 @@
           <t>FS-009645.pdf</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" t="n">
+      <c r="A58" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>FS-013354</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>Comparison of the effect of rest interval between sets and set - repetition configuration during bouts of eccentric exercise on muscle damage and inflammatory markers</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>INTERNATIONAL JOURNAL OF APPLIED EXERCISE PHYSIOLOGY</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>10.22631/ijaep.v7i1.238</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr"/>
+      <c r="H58" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.22631/ijaep.v7i1.238</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr">
+      <c r="I58" s="3" t="inlineStr"/>
+      <c r="J58" s="4" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.22631/ijaep.v7i1.238</t>
         </is>
       </c>
-      <c r="K58" s="2" t="inlineStr">
+      <c r="K58" s="4" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Comparison%20of%20the%20effect%20of%20rest%20interval%20between%20sets%20and%20set%20-%20repetition%20configuration%20during%20bouts%20of%20eccentric%20exercise%20on%20muscle%20damage%20and%20inflammatory%20markers%22</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr">
+      <c r="L58" s="3" t="inlineStr">
         <is>
           <t>FS-013354.pdf</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>PENDING_no_pdf_found</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -22071,7 +21853,11 @@
           <t>FS-003797.pdf</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -22132,7 +21918,11 @@
           <t>FS-004070.pdf</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -22193,7 +21983,11 @@
           <t>FS-003373.pdf</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -22254,7 +22048,11 @@
           <t>FS-002678.pdf</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr"/>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -22315,68 +22113,76 @@
           <t>FS-002754.pdf</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr"/>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" t="n">
+      <c r="A64" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>FS-002824</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>Exercise training, lymphocyte subsets and their cytokines production: experience of an Italian professional football team and their impact on allergy.</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>BioMed research international</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E64" s="3" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="3" t="inlineStr">
         <is>
           <t>10.1155/2014/429248</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>25050349</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H64" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1155/2014/429248</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="I64" s="4" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/25050349/</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr">
+      <c r="J64" s="4" t="inlineStr">
         <is>
           <t>https://europepmc.org/article/MED/25050349</t>
         </is>
       </c>
-      <c r="K64" s="2" t="inlineStr">
+      <c r="K64" s="4" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Exercise%20training%2C%20lymphocyte%20subsets%20and%20their%20cytokines%20production%3A%20experience%20of%20an%20Italian%20professional%20football%20team%20and%20their%20impact%20on%20allergy.%22</t>
         </is>
       </c>
-      <c r="L64" t="inlineStr">
+      <c r="L64" s="3" t="inlineStr">
         <is>
           <t>FS-002824.pdf</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr"/>
+      <c r="M64" s="3" t="inlineStr">
+        <is>
+          <t>PENDING_no_pdf_found</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -22437,7 +22243,11 @@
           <t>FS-010146.pdf</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr"/>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -22498,7 +22308,11 @@
           <t>FS-002014.pdf</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr"/>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -22559,7 +22373,11 @@
           <t>FS-001311.pdf</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr"/>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -22620,7 +22438,11 @@
           <t>FS-001124.pdf</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr"/>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -22681,7 +22503,11 @@
           <t>FS-000460.pdf</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr"/>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
D: 3 more manual PDFs registered (FS-000504 via local OCR, FS-013354, FS-002824); 67 of 68 browser-OA records retrieved, 1 pending
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fulltext_requests/library_requests_2026-10-09.xlsx
+++ b/fulltext_requests/library_requests_2026-10-09.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="library_not_OA" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="not_indexed" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="browser_OA_64_done_4_pending" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="browser_OA_67_done_1_pending" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19418,67 +19418,67 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" t="n">
         <v>1</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>FS-000504</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Immune and oxidative changes during and following the Western States Endurance Run.</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>International journal of sports medicine</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>2003</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>10.1055/s-2003-42018</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>12968214</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1055/s-2003-42018</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/12968214/</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/article/MED/12968214</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Immune%20and%20oxidative%20changes%20during%20and%20following%20the%20Western%20States%20Endurance%20Run.%22</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>FS-000504.pdf</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr">
-        <is>
-          <t>PENDING_no_pdf_found</t>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
         </is>
       </c>
     </row>
@@ -21738,59 +21738,57 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="n">
+      <c r="A58" t="n">
         <v>3</v>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>FS-013354</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>Comparison of the effect of rest interval between sets and set - repetition configuration during bouts of eccentric exercise on muscle damage and inflammatory markers</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>INTERNATIONAL JOURNAL OF APPLIED EXERCISE PHYSIOLOGY</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>10.22631/ijaep.v7i1.238</t>
         </is>
       </c>
-      <c r="G58" s="3" t="inlineStr"/>
-      <c r="H58" s="4" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.22631/ijaep.v7i1.238</t>
         </is>
       </c>
-      <c r="I58" s="3" t="inlineStr"/>
-      <c r="J58" s="4" t="inlineStr">
+      <c r="J58" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/abstract/DOI/10.22631/ijaep.v7i1.238</t>
         </is>
       </c>
-      <c r="K58" s="4" t="inlineStr">
+      <c r="K58" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Comparison%20of%20the%20effect%20of%20rest%20interval%20between%20sets%20and%20set%20-%20repetition%20configuration%20during%20bouts%20of%20eccentric%20exercise%20on%20muscle%20damage%20and%20inflammatory%20markers%22</t>
         </is>
       </c>
-      <c r="L58" s="3" t="inlineStr">
+      <c r="L58" t="inlineStr">
         <is>
           <t>FS-013354.pdf</t>
         </is>
       </c>
-      <c r="M58" s="3" t="inlineStr">
-        <is>
-          <t>PENDING_no_pdf_found</t>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
         </is>
       </c>
     </row>
@@ -22120,67 +22118,67 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n">
+      <c r="A64" t="n">
         <v>3</v>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>FS-002824</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>Exercise training, lymphocyte subsets and their cytokines production: experience of an Italian professional football team and their impact on allergy.</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>BioMed research international</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>10.1155/2014/429248</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="G64" t="inlineStr">
         <is>
           <t>25050349</t>
         </is>
       </c>
-      <c r="H64" s="4" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1155/2014/429248</t>
         </is>
       </c>
-      <c r="I64" s="4" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/25050349/</t>
         </is>
       </c>
-      <c r="J64" s="4" t="inlineStr">
+      <c r="J64" s="2" t="inlineStr">
         <is>
           <t>https://europepmc.org/article/MED/25050349</t>
         </is>
       </c>
-      <c r="K64" s="4" t="inlineStr">
+      <c r="K64" s="2" t="inlineStr">
         <is>
           <t>https://scholar.google.com/scholar?q=%22Exercise%20training%2C%20lymphocyte%20subsets%20and%20their%20cytokines%20production%3A%20experience%20of%20an%20Italian%20professional%20football%20team%20and%20their%20impact%20on%20allergy.%22</t>
         </is>
       </c>
-      <c r="L64" s="3" t="inlineStr">
+      <c r="L64" t="inlineStr">
         <is>
           <t>FS-002824.pdf</t>
         </is>
       </c>
-      <c r="M64" s="3" t="inlineStr">
-        <is>
-          <t>PENDING_no_pdf_found</t>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>retrieved_2026-10-09_by_A</t>
         </is>
       </c>
     </row>

</xml_diff>